<commit_message>
Update Config and git ignore
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BARA\Documents\UiPath\UCL_Remider_Expire\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEEC009F-194A-4C59-A94D-321A5A63CBDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BE48B10-2C80-4F24-AA4B-0D5B85119E26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="78">
   <si>
     <t>Name</t>
   </si>
@@ -153,9 +153,6 @@
   </si>
   <si>
     <t>RetryNumberAddTransactionItem</t>
-  </si>
-  <si>
-    <t>Non Production/UCL/UCL_SignedInvoiceStoring</t>
   </si>
   <si>
     <t>LogMessage_TryToGetNewLocalFile</t>
@@ -762,15 +759,15 @@
         <v>26</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" spans="1:26" ht="14.25" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1">
@@ -786,137 +783,137 @@
     </row>
     <row r="5" spans="1:26">
       <c r="A5" s="7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B5" s="4">
         <v>60</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:26" ht="14.25" customHeight="1">
       <c r="A6" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>42</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1">
       <c r="A7" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>57</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
       <c r="A8" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1">
       <c r="A9" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1">
       <c r="A10" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1">
       <c r="A11" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
       <c r="A12" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
       <c r="A13" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">
       <c r="A14" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
       <c r="A15" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1">
       <c r="A16" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="14.25" customHeight="1">
       <c r="A17" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C17" s="4" t="s">
         <v>68</v>
-      </c>
-      <c r="B17" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="315">
       <c r="A18" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="B18" s="10" t="s">
         <v>75</v>
-      </c>
-      <c r="B18" s="10" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="409.5">
       <c r="A19" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="14.25" customHeight="1"/>
@@ -2013,10 +2010,10 @@
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1">
       <c r="A10" t="s">
+        <v>39</v>
+      </c>
+      <c r="B10" t="s">
         <v>40</v>
-      </c>
-      <c r="B10" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1">
@@ -2074,7 +2071,7 @@
     </row>
     <row r="17" spans="1:3" ht="14.25" customHeight="1">
       <c r="A17" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B17">
         <v>2</v>
@@ -2082,7 +2079,7 @@
     </row>
     <row r="18" spans="1:3" ht="14.25" customHeight="1">
       <c r="A18" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B18">
         <v>2</v>
@@ -3082,7 +3079,7 @@
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="31.85546875" customWidth="1"/>
-    <col min="2" max="2" width="30.140625" customWidth="1"/>
+    <col min="2" max="2" width="43.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="60.28515625" customWidth="1"/>
     <col min="4" max="26" width="65.42578125" customWidth="1"/>
   </cols>
@@ -3125,31 +3122,156 @@
     </row>
     <row r="2" spans="1:26" ht="14.25" customHeight="1">
       <c r="A2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>49</v>
-      </c>
       <c r="C2" t="s">
-        <v>39</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A3" s="4"/>
+      <c r="A3" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A4" s="4"/>
-    </row>
-    <row r="5" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="7" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="10" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="12" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="13" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="14" spans="1:26" ht="14.25" customHeight="1"/>
+      <c r="A4" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A5" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C5" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="6" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A6" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C7" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A8" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C8" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A9" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="C9" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A10" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="C10" t="s">
+        <v>77</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A11" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C11" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="12" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A12" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C12" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="13" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A13" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C13" t="s">
+        <v>77</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="14" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A14" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C14" t="s">
+        <v>77</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="17" ht="14.25" customHeight="1"/>

</xml_diff>